<commit_message>
modifications des formules 2
</commit_message>
<xml_diff>
--- a/AutosurveillanceTemplates/Q_GRAV.xlsx
+++ b/AutosurveillanceTemplates/Q_GRAV.xlsx
@@ -6891,23 +6891,31 @@
     <row r="26" spans="2:25" ht="65.099999999999994" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.4">
       <c r="B26" s="73"/>
       <c r="C26" s="115"/>
-      <c r="D26" s="106" t="s">
-        <v>338</v>
-      </c>
-      <c r="E26" s="107" t="s">
-        <v>251</v>
-      </c>
-      <c r="F26" s="107" t="s">
-        <v>339</v>
+      <c r="D26" s="106" t="str">
+        <f>IF($D$40="Clapet","Angle simulé (°)","Hauteur simulée (mm)")</f>
+        <v>Hauteur simulée (mm)</v>
+      </c>
+      <c r="E26" s="107" t="str">
+        <f>IF($D$40="Clapet","EMT sur l'angle"&amp;CHAR(10)&amp;"(°)","EMT sur la hauteur"&amp;CHAR(10)&amp;"(mm)")</f>
+        <v>EMT sur la hauteur
+(mm)</v>
+      </c>
+      <c r="F26" s="107" t="str">
+        <f>IF($D$40="Clapet","Débit attendu / Angle simulé"&amp;CHAR(10)&amp;"(m3/h)","Débit attendu / Hauteur simulée"&amp;CHAR(10)&amp;"(m3/h)")</f>
+        <v>Débit attendu / Hauteur simulée
+(m3/h)</v>
       </c>
       <c r="G26" s="108" t="s">
         <v>250</v>
       </c>
-      <c r="H26" s="106" t="s">
-        <v>208</v>
-      </c>
-      <c r="I26" s="107" t="s">
-        <v>255</v>
+      <c r="H26" s="106" t="str">
+        <f>IF($D$40="Clapet","Angle lu (°)","Hauteur lue (mm)")</f>
+        <v>Hauteur lue (mm)</v>
+      </c>
+      <c r="I26" s="107" t="str">
+        <f>IF($D$40="Clapet","Écart"&amp;CHAR(10)&amp;"Angle lu (°)","Écart"&amp;CHAR(10)&amp;"Hauteur lue (mm)")</f>
+        <v>Écart
+Hauteur lue (mm)</v>
       </c>
       <c r="J26" s="107" t="s">
         <v>246</v>
@@ -6915,20 +6923,25 @@
       <c r="K26" s="107" t="s">
         <v>256</v>
       </c>
-      <c r="L26" s="107" t="s">
-        <v>247</v>
+      <c r="L26" s="107" t="str">
+        <f>IF($D$40="Clapet","Débit attendu / Angle lu (m3/h)","Débit attendu / Hauteur lue (m3/h)")</f>
+        <v>Débit attendu / Hauteur lue (m3/h)</v>
       </c>
       <c r="M26" s="108" t="s">
         <v>257</v>
       </c>
-      <c r="N26" s="106" t="s">
-        <v>208</v>
+      <c r="N26" s="106" t="str">
+        <f>IF($D$40="Clapet","Angle lu (°)","Hauteur lue (mm)")</f>
+        <v>Hauteur lue (mm)</v>
       </c>
       <c r="O26" s="107" t="s">
         <v>246</v>
       </c>
-      <c r="P26" s="107" t="s">
-        <v>258</v>
+      <c r="P26" s="107" t="str">
+        <f>IF($D$40="Clapet","Écart"&amp;CHAR(10)&amp;"Angle"&amp;CHAR(10)&amp;"(°)","Écart"&amp;CHAR(10)&amp;"Hauteur"&amp;CHAR(10)&amp;"(mm)")</f>
+        <v>Écart
+Hauteur
+(mm)</v>
       </c>
       <c r="Q26" s="108" t="s">
         <v>259</v>
@@ -6952,11 +6965,12 @@
       <c r="C27" s="115"/>
       <c r="D27" s="151"/>
       <c r="E27" s="100" t="str">
-        <f>IF($G$18&lt;&gt;"Mesure comparative en parallèle",IF(D27="","",IF($D$40=Critères!$AT$3,1,10)),IF(AND(H27="",N27=""),"",IF($D$40=Critères!$AT$3,1,10)))</f>
+        <f>IF($G$18&lt;&gt;"Mesure comparative en parallèle",IF(D27="","",IF($D$40="Clapet",1,10)),IF(AND(H27="",N27=""),"",IF($D$40="Clapet",1,10)))</f>
+        <v/>
       </c>
       <c r="F27" s="153"/>
       <c r="G27" s="101" t="str">
-        <f>IF($G$18&lt;&gt;"Mesure comparative en parallèle",IF(D27="","",IF(D27&lt;50,"-",IF(D27&lt;150,0.1,0.05))),IF(AND(H27="",N27=""),"",IF(AVERAGE(H27,N27)&lt;50,"-",IF(AVERAGE(H27,N27)&lt;150,0.1,0.05))))</f>
+        <f>IF($G$18&lt;&gt;"Mesure comparative en parallèle",IF(D27="","",IF($D$40="Clapet",0.1,IF(D27&lt;50,"-",IF(D27&lt;150,0.1,0.05)))),IF(AND(H27="",N27=""),"",IF($D$40="Clapet",0.1,IF(AVERAGE(H27,N27)&lt;50,"-",IF(AVERAGE(H27,N27)&lt;150,0.1,0.05)))))</f>
         <v/>
       </c>
       <c r="H27" s="151"/>
@@ -7003,11 +7017,12 @@
       <c r="C28" s="115"/>
       <c r="D28" s="151"/>
       <c r="E28" s="100" t="str">
-        <f>IF($G$18&lt;&gt;"Mesure comparative en parallèle",IF(D28="","",IF($D$40=Critères!$AT$3,1,10)),IF(AND(H28="",N28=""),"",IF($D$40=Critères!$AT$3,1,10)))</f>
+        <f>IF($G$18&lt;&gt;"Mesure comparative en parallèle",IF(D28="","",IF($D$40="Clapet",1,10)),IF(AND(H28="",N28=""),"",IF($D$40="Clapet",1,10)))</f>
+        <v/>
       </c>
       <c r="F28" s="153"/>
       <c r="G28" s="101" t="str">
-        <f t="shared" ref="G28:G30" si="0">IF($G$18&lt;&gt;"Mesure comparative en parallèle",IF(D28="","",IF(D28&lt;50,"-",IF(D28&lt;150,0.1,0.05))),IF(AND(H28="",N28=""),"",IF(AVERAGE(H28,N28)&lt;50,"-",IF(AVERAGE(H28,N28)&lt;150,0.1,0.05))))</f>
+        <f>IF($G$18&lt;&gt;"Mesure comparative en parallèle",IF(D28="","",IF($D$40="Clapet",0.1,IF(D28&lt;50,"-",IF(D28&lt;150,0.1,0.05)))),IF(AND(H28="",N28=""),"",IF($D$40="Clapet",0.1,IF(AVERAGE(H28,N28)&lt;50,"-",IF(AVERAGE(H28,N28)&lt;150,0.1,0.05)))))</f>
         <v/>
       </c>
       <c r="H28" s="151"/>
@@ -7040,13 +7055,13 @@
       <c r="T28" s="116"/>
       <c r="U28" s="74"/>
       <c r="W28" s="236">
-        <f t="shared" ref="W28:W30" si="4">IF($G$18="Mesure comparative en parallèle",IF(AND(ISNUMBER(P28),ISNUMBER(E28)),IF(ABS(P28)&gt;E28,1,0),0),IF(AND(ISNUMBER(I28),ISNUMBER(E28)),IF(ABS(I28)&gt;E28,1,0),0))</f>
+        <f>IF($G$18="Mesure comparative en parallèle",IF(AND(ISNUMBER(P28),ISNUMBER(E28)),IF(ABS(P28)&gt;E28,1,0),0),IF(AND(ISNUMBER(I28),ISNUMBER(E28)),IF(ABS(I28)&gt;E28,1,0),0))</f>
       </c>
       <c r="X28" s="236">
-        <f t="shared" ref="X28:X30" si="5">IF($G$18="Mesure comparative en parallèle",0,IF(AND(ISNUMBER(K28),ISNUMBER(G28)),IF(ABS(K28)&gt;G28,1,0),0))</f>
+        <f>IF($G$18="Mesure comparative en parallèle",0,IF(AND(ISNUMBER(K28),ISNUMBER(G28)),IF(ABS(K28)&gt;G28,1,0),0))</f>
       </c>
       <c r="Y28" s="236">
-        <f t="shared" ref="Y28:Y30" si="6">IF($G$18="Mesure comparative en parallèle",IF(AND(ISNUMBER(Q28),ISNUMBER(G28)),IF(ABS(Q28)&gt;G28,1,0),0),0)</f>
+        <f>IF($G$18="Mesure comparative en parallèle",IF(AND(ISNUMBER(Q28),ISNUMBER(G28)),IF(ABS(Q28)&gt;G28,1,0),0),0)</f>
       </c>
     </row>
     <row r="29" spans="2:25" ht="20.100000000000001" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.4">
@@ -7054,11 +7069,12 @@
       <c r="C29" s="115"/>
       <c r="D29" s="151"/>
       <c r="E29" s="100" t="str">
-        <f>IF($G$18&lt;&gt;"Mesure comparative en parallèle",IF(D29="","",IF($D$40=Critères!$AT$3,1,10)),IF(AND(H29="",N29=""),"",IF($D$40=Critères!$AT$3,1,10)))</f>
+        <f>IF($G$18&lt;&gt;"Mesure comparative en parallèle",IF(D29="","",IF($D$40="Clapet",1,10)),IF(AND(H29="",N29=""),"",IF($D$40="Clapet",1,10)))</f>
+        <v/>
       </c>
       <c r="F29" s="153"/>
       <c r="G29" s="101" t="str">
-        <f t="shared" si="0"/>
+        <f>IF($G$18&lt;&gt;"Mesure comparative en parallèle",IF(D29="","",IF($D$40="Clapet",0.1,IF(D29&lt;50,"-",IF(D29&lt;150,0.1,0.05)))),IF(AND(H29="",N29=""),"",IF($D$40="Clapet",0.1,IF(AVERAGE(H29,N29)&lt;50,"-",IF(AVERAGE(H29,N29)&lt;150,0.1,0.05)))))</f>
         <v/>
       </c>
       <c r="H29" s="151"/>
@@ -7091,16 +7107,13 @@
       <c r="T29" s="116"/>
       <c r="U29" s="74"/>
       <c r="W29" s="236">
-        <f t="shared" si="4"/>
-        <v>0</v>
+        <f>IF($G$18="Mesure comparative en parallèle",IF(AND(ISNUMBER(P29),ISNUMBER(E29)),IF(ABS(P29)&gt;E29,1,0),0),IF(AND(ISNUMBER(I29),ISNUMBER(E29)),IF(ABS(I29)&gt;E29,1,0),0))</f>
       </c>
       <c r="X29" s="236">
-        <f t="shared" si="5"/>
-        <v>0</v>
+        <f>IF($G$18="Mesure comparative en parallèle",0,IF(AND(ISNUMBER(K29),ISNUMBER(G29)),IF(ABS(K29)&gt;G29,1,0),0))</f>
       </c>
       <c r="Y29" s="236">
-        <f t="shared" si="6"/>
-        <v>0</v>
+        <f>IF($G$18="Mesure comparative en parallèle",IF(AND(ISNUMBER(Q29),ISNUMBER(G29)),IF(ABS(Q29)&gt;G29,1,0),0),0)</f>
       </c>
     </row>
     <row r="30" spans="2:25" ht="20.100000000000001" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.4">
@@ -7108,11 +7121,12 @@
       <c r="C30" s="115"/>
       <c r="D30" s="152"/>
       <c r="E30" s="146" t="str">
-        <f>IF($G$18&lt;&gt;"Mesure comparative en parallèle",IF(D30="","",IF($D$40=Critères!$AT$3,1,10)),IF(AND(H30="",N30=""),"",IF($D$40=Critères!$AT$3,1,10)))</f>
+        <f>IF($G$18&lt;&gt;"Mesure comparative en parallèle",IF(D30="","",IF($D$40="Clapet",1,10)),IF(AND(H30="",N30=""),"",IF($D$40="Clapet",1,10)))</f>
+        <v/>
       </c>
       <c r="F30" s="154"/>
       <c r="G30" s="147" t="str">
-        <f t="shared" si="0"/>
+        <f>IF($G$18&lt;&gt;"Mesure comparative en parallèle",IF(D30="","",IF($D$40="Clapet",0.1,IF(D30&lt;50,"-",IF(D30&lt;150,0.1,0.05)))),IF(AND(H30="",N30=""),"",IF($D$40="Clapet",0.1,IF(AVERAGE(H30,N30)&lt;50,"-",IF(AVERAGE(H30,N30)&lt;150,0.1,0.05)))))</f>
         <v/>
       </c>
       <c r="H30" s="152"/>
@@ -7145,16 +7159,13 @@
       <c r="T30" s="116"/>
       <c r="U30" s="74"/>
       <c r="W30" s="236">
-        <f t="shared" si="4"/>
-        <v>0</v>
+        <f>IF($G$18="Mesure comparative en parallèle",IF(AND(ISNUMBER(P30),ISNUMBER(E30)),IF(ABS(P30)&gt;E30,1,0),0),IF(AND(ISNUMBER(I30),ISNUMBER(E30)),IF(ABS(I30)&gt;E30,1,0),0))</f>
       </c>
       <c r="X30" s="236">
-        <f t="shared" si="5"/>
-        <v>0</v>
+        <f>IF($G$18="Mesure comparative en parallèle",0,IF(AND(ISNUMBER(K30),ISNUMBER(G30)),IF(ABS(K30)&gt;G30,1,0),0))</f>
       </c>
       <c r="Y30" s="236">
-        <f t="shared" si="6"/>
-        <v>0</v>
+        <f>IF($G$18="Mesure comparative en parallèle",IF(AND(ISNUMBER(Q30),ISNUMBER(G30)),IF(ABS(Q30)&gt;G30,1,0),0),0)</f>
       </c>
     </row>
     <row r="31" spans="2:25" ht="20.100000000000001" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.4">
@@ -7180,12 +7191,15 @@
       <c r="U31" s="74"/>
       <c r="W31" s="236" t="str">
         <f>IF(IF($G$18="Mesure comparative en parallèle",COUNT(P27:P30),COUNT(I27:I30))&gt;0,IF(SUM(W27:W30)&gt;0,"Non validé","Validé"),"Non contrôlé")</f>
+        <v/>
       </c>
       <c r="X31" s="236" t="str">
         <f>IF($G$18="Mesure comparative en parallèle","-",IF(SUMPRODUCT(ISNUMBER(K27:K30)*ISNUMBER(G27:G30))&gt;0,IF(SUM(X27:X30)&gt;0,"Non validé","Validé"),"Non contrôlé"))</f>
+        <v/>
       </c>
       <c r="Y31" s="236" t="str">
         <f>IF($G$18="Mesure comparative en parallèle",IF(SUMPRODUCT(ISNUMBER(Q27:Q30)*ISNUMBER(G27:G30))&gt;0,IF(SUM(Y27:Y30)&gt;0,"Non validé","Validé"),"Non contrôlé"),"-")</f>
+        <v/>
       </c>
     </row>
     <row r="32" spans="2:25" ht="20.100000000000001" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.4">
@@ -7215,6 +7229,7 @@
       <c r="U32" s="74"/>
       <c r="X32" s="236" t="str">
         <f>IF($G$18="Mesure comparative en parallèle",Y31,X31)</f>
+        <v/>
       </c>
     </row>
     <row r="33" spans="2:37" s="85" customFormat="1" ht="20.100000000000001" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.4">
@@ -7795,7 +7810,7 @@
       <c r="N48" s="267"/>
       <c r="O48" s="268"/>
       <c r="P48" s="264" t="str">
-        <f>IF(E48="-","Non applicable",IF(D40=Critères!BB3,"Non contrôlé",W31))</f>
+        <f>IF(E48="-","Non applicable",IF(D40="Détecteur de surverse","Non contrôlé",W31))</f>
       </c>
       <c r="Q48" s="265"/>
       <c r="R48" s="93">
@@ -7837,7 +7852,8 @@
       <c r="N49" s="267"/>
       <c r="O49" s="268"/>
       <c r="P49" s="264" t="str">
-        <f>IF(E49="-","Non applicable",IF(D40=Critères!BB3,"Non contrôlé",X32))</f>
+        <f>IF(E49="-","Non applicable",IF(D40="Détecteur de surverse","Non contrôlé",X32))</f>
+        <v/>
       </c>
       <c r="Q49" s="265"/>
       <c r="R49" s="93">

</xml_diff>